<commit_message>
streamlit app initial commit
</commit_message>
<xml_diff>
--- a/ΕΝΗΜΕΡΩΤΙΚΑ_ΣΗΜΕΙΩΜΑΤΑ/2026-01/XLSX/ΕΝΗΜΕΡΩΤΙΚΟ_ΣΗΜΕΙΩΜΑ_AMYKLAION_ENERGY_IKE_2026-01.xlsx
+++ b/ΕΝΗΜΕΡΩΤΙΚΑ_ΣΗΜΕΙΩΜΑΤΑ/2026-01/XLSX/ΕΝΗΜΕΡΩΤΙΚΟ_ΣΗΜΕΙΩΜΑ_AMYKLAION_ENERGY_IKE_2026-01.xlsx
@@ -699,7 +699,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -974,7 +974,13 @@
     <xf numFmtId="168" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="11" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="12" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="12" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="12" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2832,7 +2838,7 @@
     <row r="6" ht="60.75" customFormat="1" customHeight="1" s="10">
       <c r="B6" s="80" t="inlineStr">
         <is>
-          <t>13/02/26</t>
+          <t>06/03/26</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -3521,36 +3527,36 @@
         </is>
       </c>
       <c r="D40" s="25" t="n">
-        <v>0</v>
+        <v>2094.44</v>
       </c>
       <c r="E40" s="25" t="n">
-        <v>0</v>
+        <v>178.647196</v>
       </c>
       <c r="F40" s="25" t="n">
-        <v>0</v>
+        <v>2.09</v>
       </c>
       <c r="G40" s="92" t="n">
-        <v>0</v>
+        <v>85.3</v>
       </c>
       <c r="H40" s="93" t="n"/>
     </row>
     <row r="41" ht="28.5" customHeight="1" s="76" thickBot="1">
-      <c r="C41" s="29" t="inlineStr">
+      <c r="C41" s="94" t="inlineStr">
         <is>
           <t>Σύνολο</t>
         </is>
       </c>
-      <c r="D41" s="30" t="n">
-        <v>34817.38</v>
-      </c>
-      <c r="E41" s="30" t="n">
-        <v>2814.66</v>
-      </c>
-      <c r="F41" s="30" t="n">
-        <v>34.84</v>
-      </c>
-      <c r="G41" s="94" t="n">
-        <v>80.84</v>
+      <c r="D41" s="95" t="n">
+        <v>36911.82</v>
+      </c>
+      <c r="E41" s="95" t="n">
+        <v>2993.3</v>
+      </c>
+      <c r="F41" s="95" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="G41" s="96" t="n">
+        <v>81.09</v>
       </c>
       <c r="H41" s="93" t="n"/>
     </row>
@@ -3559,7 +3565,7 @@
       <c r="D42" s="33" t="n"/>
       <c r="E42" s="33" t="n"/>
       <c r="F42" s="34" t="n"/>
-      <c r="G42" s="95" t="n"/>
+      <c r="G42" s="97" t="n"/>
       <c r="H42" s="93" t="n"/>
     </row>
     <row r="43" ht="49" customHeight="1" s="76" thickBot="1">
@@ -3573,16 +3579,16 @@
           <t>Ανάλυση Χρεώσεων και Υπηρεσίων ΦοΣΕ</t>
         </is>
       </c>
-      <c r="C44" s="96" t="n"/>
-      <c r="D44" s="97" t="n"/>
+      <c r="C44" s="98" t="n"/>
+      <c r="D44" s="99" t="n"/>
       <c r="E44" s="18" t="n"/>
-      <c r="F44" s="98" t="inlineStr">
+      <c r="F44" s="100" t="inlineStr">
         <is>
           <t>Υπολογισμός προς καταβολή</t>
         </is>
       </c>
-      <c r="G44" s="96" t="n"/>
-      <c r="H44" s="99" t="n"/>
+      <c r="G44" s="98" t="n"/>
+      <c r="H44" s="101" t="n"/>
       <c r="I44" s="45" t="n"/>
     </row>
     <row r="45" ht="36" customHeight="1" s="76">
@@ -3592,7 +3598,7 @@
         </is>
       </c>
       <c r="C45" s="83" t="n"/>
-      <c r="D45" s="100" t="n">
+      <c r="D45" s="102" t="n">
         <v>1</v>
       </c>
       <c r="E45" s="44" t="n"/>
@@ -3602,8 +3608,8 @@
         </is>
       </c>
       <c r="G45" s="83" t="n"/>
-      <c r="H45" s="101" t="n">
-        <v>34.82</v>
+      <c r="H45" s="103" t="n">
+        <v>36.91</v>
       </c>
       <c r="I45" s="45" t="n"/>
     </row>
@@ -3613,9 +3619,9 @@
           <t>Σύνολο (€)</t>
         </is>
       </c>
-      <c r="C46" s="102" t="n"/>
-      <c r="D46" s="103" t="n">
-        <v>34.84</v>
+      <c r="C46" s="104" t="n"/>
+      <c r="D46" s="105" t="n">
+        <v>36.93</v>
       </c>
       <c r="E46" s="41" t="n"/>
       <c r="F46" s="60" t="inlineStr">
@@ -3624,8 +3630,8 @@
         </is>
       </c>
       <c r="G46" s="83" t="n"/>
-      <c r="H46" s="101" t="n">
-        <v>2814.66</v>
+      <c r="H46" s="103" t="n">
+        <v>2993.3</v>
       </c>
       <c r="I46" s="45" t="n"/>
     </row>
@@ -3664,7 +3670,7 @@
           <t xml:space="preserve">Συνολικό Ποσό προς καταβολή </t>
         </is>
       </c>
-      <c r="G49" s="102" t="n"/>
+      <c r="G49" s="104" t="n"/>
       <c r="H49" s="48">
         <f>H46+H47+H48</f>
         <v/>
@@ -3685,16 +3691,16 @@
           <t>Στοιχεία Τράπεζας</t>
         </is>
       </c>
-      <c r="C51" s="96" t="n"/>
-      <c r="D51" s="97" t="n"/>
+      <c r="C51" s="98" t="n"/>
+      <c r="D51" s="99" t="n"/>
       <c r="E51" s="41" t="n"/>
-      <c r="F51" s="98" t="inlineStr">
+      <c r="F51" s="100" t="inlineStr">
         <is>
           <t>Υπολογισμός Τιμολόγησης</t>
         </is>
       </c>
-      <c r="G51" s="96" t="n"/>
-      <c r="H51" s="99" t="n"/>
+      <c r="G51" s="98" t="n"/>
+      <c r="H51" s="101" t="n"/>
       <c r="I51" s="45" t="n"/>
     </row>
     <row r="52" ht="25.25" customHeight="1" s="76">
@@ -3703,12 +3709,12 @@
           <t xml:space="preserve"> ΙΒΑΝ</t>
         </is>
       </c>
-      <c r="C52" s="104" t="inlineStr">
+      <c r="C52" s="106" t="inlineStr">
         <is>
           <t>GR6803400150015004285091197</t>
         </is>
       </c>
-      <c r="D52" s="105" t="n"/>
+      <c r="D52" s="107" t="n"/>
       <c r="E52" s="41" t="n"/>
       <c r="F52" s="60" t="inlineStr">
         <is>
@@ -3728,12 +3734,12 @@
           <t xml:space="preserve"> Ημερομηνία</t>
         </is>
       </c>
-      <c r="C53" s="106" t="inlineStr">
-        <is>
-          <t>15/02/26</t>
-        </is>
-      </c>
-      <c r="D53" s="107" t="n"/>
+      <c r="C53" s="108" t="inlineStr">
+        <is>
+          <t>08/03/26</t>
+        </is>
+      </c>
+      <c r="D53" s="109" t="n"/>
       <c r="E53" s="41" t="n"/>
       <c r="F53" s="60" t="inlineStr">
         <is>
@@ -3757,7 +3763,7 @@
           <t xml:space="preserve">ΓΕΝΙΚΟ ΣΥΝΟΛΟ </t>
         </is>
       </c>
-      <c r="G54" s="102" t="n"/>
+      <c r="G54" s="104" t="n"/>
       <c r="H54" s="43">
         <f>H52+H53</f>
         <v/>
@@ -3766,7 +3772,7 @@
     </row>
     <row r="55" ht="28.75" customHeight="1" s="76"/>
     <row r="56" ht="38.25" customHeight="1" s="76">
-      <c r="B56" s="108" t="inlineStr">
+      <c r="B56" s="110" t="inlineStr">
         <is>
           <t>Σημείωση: Το τελικό ποσό πίστωσης παραγωγού προκύπτει από το άθροισμα των γινομένων της παραγόμενης ενέργειας επί της αντίστοιχης Τιμής Εκκαθάρισης Αγοράς Επόμενης Ημέρας ανά 15', αφαιρώντας την πληρωμή υπηρεσιών ΦοΣΕ και Διαχειριστικών εξόδων. Οι πληρωμές της GREEN VALUE Α.Ε. πραγματοποιουνται εντός 2 εργάσιμων ημερών μετά την παραλαβή του ενημερωτικού σημειώματος.</t>
         </is>

</xml_diff>